<commit_message>
Registers: Open Items v0.6 (OI-18, OI-19), Technical Debt Register v0.2 (TD-004), Defect Register v0.3 (DEF-017; DEF-014/015 observed absence), Decision Log v0.8 (DEC-019); v0.2 and v0.7 moved to Outdated
</commit_message>
<xml_diff>
--- a/docs/Requirements/Open Items/Open_Items_v0.6.xlsx
+++ b/docs/Requirements/Open Items/Open_Items_v0.6.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huawei\Desktop\SEN381\Ticketing-System\docs\Requirements\Open Items\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{975CC829-C284-4991-B3D5-A10599F1EC14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0676F79-B3E3-4F25-BE7E-233123A13534}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13286" yWindow="0" windowWidth="13543" windowHeight="17914" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="26949" windowHeight="18034" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Open Items" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="118">
   <si>
     <t>Open Items &amp; Assumptions</t>
   </si>
@@ -328,9 +328,6 @@
     <t>OI-01, OI-02, OI-03 and OI-08 are requirements work exposing gaps and instability in the scope baseline. That is traceability doing its job: it is only useful if it can fail. Raise them as GitHub issues against Member A under the DEC-008 branching model rather than resolving them silently here. OI-09 and OI-11 are closed by being recorded: they document deliberate non-derivations so that a missing requirement reads as a decision.</t>
   </si>
   <si>
-    <t>Gaps, derived requirements and unvalidated figures carried by this baseline. Recorded rather than resolved by invention — Master Brief s.23 values honest limitations above unsupported claims of completeness | Version 0.6 (12/10/2026). Adds OI-17 (the read endpoint refuses the whole read of a security-category request to non-Security-Officer staff, which is wider than FR-1.5's three restricted fields), raised by E. Lindsay; OI-01 to OI-16 unchanged. Version 0.5 (30/09/2026). Adds OI-16 (FR-1.5 against FR-3.5/FR-3.6: whether a requester may see their own description on a security-category request), raised by E. Lindsay; OI-01 to OI-15 unchanged. Version 0.4 (30/09/2026). Adds OI-14 (reportingCounts reconciliation, owner R. van der Merwe for M3) and OI-15 (transition model confirmation, including whether a reopened-then-resolved request satisfies FR-6.5), both raised in PR #62 (E. Lindsay) and its review (R. van der Merwe). OI-01 to OI-13 are unchanged from v0.3. Version 0.3 (29/09/2026). Consolidates the M2 updates drafted by E. Lindsay (OI-05 closed; OI-06 escalated; OI-07, OI-10 updated; OI-12 raised), first committed inside the file named Open_Items_v0.2 (archived in Outdated/ and carrying those v0.3 labels), with the DEC-017 and storage updates by R. van der Merwe (OI-06 closed, OI-10 reduced, OI-13 raised). No separately committed v0.2 content exists in the repository.</t>
-  </si>
-  <si>
     <t>OI-17</t>
   </si>
   <si>
@@ -344,6 +341,39 @@
   </si>
   <si>
     <t>Raised 12/10/2026 by E. Lindsay. Related: OI-15, OI-16, CFL-002, Condition C-01</t>
+  </si>
+  <si>
+    <t>OI-18</t>
+  </si>
+  <si>
+    <t>FR-6.6 requires closing or rejecting “with a recorded reason”. AC-FR-6.6 tests a transition “submitted without a reason, and then resubmitted with one”, and DEC-015 §4 maps “reason missing on close/reject” to 422. None of them says whether a blank or whitespace-only reason is “a reason”. The implementation treats any non-empty string as a recorded reason (statusTransitionService.js, hasReason: Boolean(reason)), so a reason of a single space is accepted and stored. The recorded reason is what FR-3.4 feeds back to the requester on rejection (FR-6.6 note). Not decided from the code.</t>
+  </si>
+  <si>
+    <t>FR-6.6, AC-FR-6.6, FR-3.4, DEC-015 §4, src/services/statusTransitionService.js, src/domain/requestStatus.js (REASON_REQUIRED)</t>
+  </si>
+  <si>
+    <t>Team decides whether a reason must contain non-whitespace text. If yes: a controlled change to AC-FR-6.6 (or its measure) stating it, a defect for the current behaviour, a server-side check returning 422 as for a missing reason, and a negative-verified test. If no: record that any non-empty string satisfies FR-6.6, and close.</t>
+  </si>
+  <si>
+    <t>Raised 12/10/2026 by E. Lindsay. Related: FR-3.4, DEC-015</t>
+  </si>
+  <si>
+    <t>OI-19</t>
+  </si>
+  <si>
+    <t>DEC-003 v0.2’s environment map names the test environment “civicconnect-test” (Atlas project / cluster column). The integration-test guard (tests/integration/_harness.js, PR #88) runs only when the host in MONGODB_URI contains “civicconnecttest”, with no hyphen, and the test cluster’s actual host does contain that unhyphenated spelling: a read-only run on 2026-10-12 used the real test connection string and passed the same host check (docs/evidence/M3-indexes/listIndexes_refused_civicconnect-app.txt; the host itself is not recorded). The run evidence (docs/evidence/M3_API_Test_Run.txt) gives the project as “CivicConnect-Test”. So the record has one spelling and the environment and code use another. DEC-003’s column also doesn’t separate the Atlas project name from the cluster name, and the host comes from the cluster name. A guard written from DEC-003’s spelling would refuse the real test cluster; one written from the host doesn’t trace to the record. The URI itself is not in the repository and was not read.</t>
+  </si>
+  <si>
+    <t>DEC-003 (environment map, Test row), tests/integration/_harness.js (TEST_CLUSTER_MARKER), M3 API Test Specification §3.2, docs/evidence/M3_API_Test_Run.txt, the planned E2E guard (DEC-019); related: DEF-006</t>
+  </si>
+  <si>
+    <t>Record the test environment’s Atlas project name and cluster name separately, as they exist, in a new DEC-003 version (the deploy-procedure gap from DEC-019 and the index step from TD-004 could go in the same version). Then the guard’s marker cites that record, and the E2E guard uses the same value. If the cluster is renamed instead, the guard and the evidence change with it.</t>
+  </si>
+  <si>
+    <t>Raised 12/10/2026 by E. Lindsay. Related: R. van der Merwe (DEC-003 owner), DEF-006, DEC-019</t>
+  </si>
+  <si>
+    <t>Gaps, derived requirements and unvalidated figures carried by this baseline. Recorded rather than resolved by invention — Master Brief s.23 values honest limitations above unsupported claims of completeness | Version 0.6 (12/10/2026). Adds OI-17 (the read endpoint refuses the whole read of a security-category request to non-Security-Officer staff, which is wider than FR-1.5's three restricted fields), OI-18 (whether a blank or whitespace-only reason counts as a recorded reason under FR-6.6) and OI-19 (DEC-003 names the test environment's Atlas project civicconnect-test, but the test cluster's host and the integration-test guard use civicconnecttest), all raised by E. Lindsay; OI-01 to OI-16 unchanged. Version 0.5 (30/09/2026). Adds OI-16 (FR-1.5 against FR-3.5/FR-3.6: whether a requester may see their own description on a security-category request), raised by E. Lindsay; OI-01 to OI-15 unchanged. Version 0.4 (30/09/2026). Adds OI-14 (reportingCounts reconciliation, owner R. van der Merwe for M3) and OI-15 (transition model confirmation, including whether a reopened-then-resolved request satisfies FR-6.5), both raised in PR #62 (E. Lindsay) and its review (R. van der Merwe). OI-01 to OI-13 are unchanged from v0.3. Version 0.3 (29/09/2026). Consolidates the M2 updates drafted by E. Lindsay (OI-05 closed; OI-06 escalated; OI-07, OI-10 updated; OI-12 raised), first committed inside the file named Open_Items_v0.2 (archived in Outdated/ and carrying those v0.3 labels), with the DEC-017 and storage updates by R. van der Merwe (OI-06 closed, OI-10 reduced, OI-13 raised). No separately committed v0.2 content exists in the repository.</t>
   </si>
 </sst>
 </file>
@@ -488,7 +518,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -496,14 +526,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -531,6 +553,15 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -798,7 +829,7 @@
   <sheetPr>
     <tabColor rgb="FF0F4761"/>
   </sheetPr>
-  <dimension ref="B1:H22"/>
+  <dimension ref="B1:H24"/>
   <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="2.3046875" customWidth="1"/>
@@ -812,26 +843,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:8" ht="24.45" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-    </row>
-    <row r="2" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+    </row>
+    <row r="2" spans="2:8" ht="82.3" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B2" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
     </row>
     <row r="4" spans="2:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B4" s="1" t="s">
@@ -856,8 +887,8 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="2:8" ht="54" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B5" s="14" t="s">
+    <row r="5" spans="2:8" ht="42.45" x14ac:dyDescent="0.4">
+      <c r="B5" s="10" t="s">
         <v>8</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -866,7 +897,7 @@
       <c r="D5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="5" t="s">
         <v>11</v>
       </c>
       <c r="F5" s="2" t="s">
@@ -879,8 +910,8 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="2:8" ht="41.25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B6" s="14" t="s">
+    <row r="6" spans="2:8" ht="42.45" x14ac:dyDescent="0.4">
+      <c r="B6" s="10" t="s">
         <v>15</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -889,7 +920,7 @@
       <c r="D6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="5" t="s">
         <v>18</v>
       </c>
       <c r="F6" s="2" t="s">
@@ -902,8 +933,8 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="2:8" ht="54" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B7" s="14" t="s">
+    <row r="7" spans="2:8" ht="42.45" x14ac:dyDescent="0.4">
+      <c r="B7" s="10" t="s">
         <v>20</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -912,7 +943,7 @@
       <c r="D7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="5" t="s">
         <v>22</v>
       </c>
       <c r="F7" s="2" t="s">
@@ -925,8 +956,8 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="2:8" ht="66.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B8" s="14" t="s">
+    <row r="8" spans="2:8" ht="56.6" x14ac:dyDescent="0.4">
+      <c r="B8" s="10" t="s">
         <v>24</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -935,7 +966,7 @@
       <c r="D8" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="5" t="s">
         <v>27</v>
       </c>
       <c r="F8" s="2" t="s">
@@ -948,8 +979,8 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="2:8" ht="41.25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B9" s="14" t="s">
+    <row r="9" spans="2:8" ht="84.9" x14ac:dyDescent="0.4">
+      <c r="B9" s="10" t="s">
         <v>31</v>
       </c>
       <c r="C9" s="2" t="s">
@@ -958,7 +989,7 @@
       <c r="D9" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="5" t="s">
         <v>34</v>
       </c>
       <c r="F9" s="2" t="s">
@@ -971,8 +1002,8 @@
         <v>37</v>
       </c>
     </row>
-    <row r="10" spans="2:8" ht="66.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B10" s="14" t="s">
+    <row r="10" spans="2:8" ht="240.45" x14ac:dyDescent="0.4">
+      <c r="B10" s="10" t="s">
         <v>38</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -981,7 +1012,7 @@
       <c r="D10" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="5" t="s">
         <v>41</v>
       </c>
       <c r="F10" s="2" t="s">
@@ -994,8 +1025,8 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="2:8" ht="54" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B11" s="14" t="s">
+    <row r="11" spans="2:8" ht="84.9" x14ac:dyDescent="0.4">
+      <c r="B11" s="10" t="s">
         <v>44</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -1004,7 +1035,7 @@
       <c r="D11" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="5" t="s">
         <v>46</v>
       </c>
       <c r="F11" s="2" t="s">
@@ -1017,8 +1048,8 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="2:8" ht="79.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="14" t="s">
+    <row r="12" spans="2:8" ht="70.75" x14ac:dyDescent="0.4">
+      <c r="B12" s="10" t="s">
         <v>49</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -1027,7 +1058,7 @@
       <c r="D12" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="E12" s="5" t="s">
         <v>52</v>
       </c>
       <c r="F12" s="2" t="s">
@@ -1040,8 +1071,8 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="2:8" ht="54" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B13" s="14" t="s">
+    <row r="13" spans="2:8" ht="56.6" x14ac:dyDescent="0.4">
+      <c r="B13" s="10" t="s">
         <v>55</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -1050,7 +1081,7 @@
       <c r="D13" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="5" t="s">
         <v>58</v>
       </c>
       <c r="F13" s="2" t="s">
@@ -1063,8 +1094,8 @@
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="2:8" ht="66.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B14" s="14" t="s">
+    <row r="14" spans="2:8" ht="155.6" x14ac:dyDescent="0.4">
+      <c r="B14" s="10" t="s">
         <v>61</v>
       </c>
       <c r="C14" s="2" t="s">
@@ -1073,7 +1104,7 @@
       <c r="D14" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="E14" s="5" t="s">
         <v>64</v>
       </c>
       <c r="F14" s="2" t="s">
@@ -1086,8 +1117,8 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="2:8" ht="66.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B15" s="14" t="s">
+    <row r="15" spans="2:8" ht="56.6" x14ac:dyDescent="0.4">
+      <c r="B15" s="10" t="s">
         <v>67</v>
       </c>
       <c r="C15" s="2" t="s">
@@ -1096,7 +1127,7 @@
       <c r="D15" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="5" t="s">
         <v>69</v>
       </c>
       <c r="F15" s="2" t="s">
@@ -1109,159 +1140,205 @@
         <v>60</v>
       </c>
     </row>
-    <row r="16" spans="2:8" ht="66.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B16" s="15" t="s">
+    <row r="16" spans="2:8" ht="99" x14ac:dyDescent="0.4">
+      <c r="B16" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="E16" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="G16" s="7" t="s">
+      <c r="G16" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="H16" s="7" t="s">
+      <c r="H16" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B17" s="8" t="s">
+    <row r="17" spans="2:8" ht="102" x14ac:dyDescent="0.4">
+      <c r="B17" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="D17" s="12" t="s">
+      <c r="D17" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="E17" s="13" t="s">
+      <c r="E17" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="F17" s="12" t="s">
+      <c r="F17" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="G17" s="12" t="s">
+      <c r="G17" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="H17" s="12" t="s">
+      <c r="H17" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="2:8" ht="105" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B18" s="8" t="s">
+    <row r="18" spans="2:8" ht="102" x14ac:dyDescent="0.4">
+      <c r="B18" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="C18" s="11" t="s">
+      <c r="C18" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="D18" s="12" t="s">
+      <c r="D18" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="E18" s="13" t="s">
+      <c r="E18" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="F18" s="12" t="s">
+      <c r="F18" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="G18" s="12" t="s">
+      <c r="G18" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="H18" s="12" t="s">
+      <c r="H18" s="8" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="19" spans="2:8" ht="150" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B19" s="8" t="s">
+    <row r="19" spans="2:8" ht="204" x14ac:dyDescent="0.4">
+      <c r="B19" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="C19" s="12" t="s">
+      <c r="C19" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="D19" s="12" t="s">
+      <c r="D19" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="E19" s="13" t="s">
+      <c r="E19" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="F19" s="12" t="s">
+      <c r="F19" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="G19" s="12" t="s">
+      <c r="G19" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="H19" s="12" t="s">
+      <c r="H19" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="2:8" ht="105" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B20" s="8" t="s">
+    <row r="20" spans="2:8" ht="72.900000000000006" x14ac:dyDescent="0.4">
+      <c r="B20" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="C20" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="D20" s="12" t="s">
+      <c r="D20" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="E20" s="13" t="s">
+      <c r="E20" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="F20" s="12" t="s">
+      <c r="F20" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="G20" s="12" t="s">
+      <c r="G20" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="H20" s="12" t="s">
+      <c r="H20" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="2:8" ht="105" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B21" s="8" t="s">
+    <row r="21" spans="2:8" ht="131.15" x14ac:dyDescent="0.4">
+      <c r="B21" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="D21" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="C21" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="D21" s="12" t="s">
+      <c r="E21" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="E21" s="13" t="s">
+      <c r="F21" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="F21" s="12" t="s">
+      <c r="G21" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="G21" s="12" t="s">
+      <c r="H21" s="8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" ht="102" x14ac:dyDescent="0.4">
+      <c r="B22" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="H21" s="12" t="s">
+      <c r="C22" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="G22" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="H22" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="22" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B22" s="5" t="s">
+    <row r="23" spans="2:8" ht="189.45" x14ac:dyDescent="0.4">
+      <c r="B23" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="G23" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="H23" s="8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.4">
+      <c r="B24" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="13"/>
+      <c r="G24" s="13"/>
+      <c r="H24" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B22:H22"/>
+    <mergeCell ref="B24:H24"/>
     <mergeCell ref="B2:H2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>